<commit_message>
feat: modern UI design, browser webcam scanner and dynamic face enrollment
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.44140625" customWidth="1" min="1" max="3"/>
@@ -574,6 +574,40 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>nihar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>16:39:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Subodh</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16:49:04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs: add comprehensive README with team contributions, architecture diagram, and setup guide
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.44140625" customWidth="1" min="1" max="3"/>
@@ -608,6 +608,23 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>nihar</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17:05:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>